<commit_message>
New versions of field results
</commit_message>
<xml_diff>
--- a/Field-trails/2025-11-05-Pig-Slurry/DFC overview pig.xlsx
+++ b/Field-trails/2025-11-05-Pig-Slurry/DFC overview pig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Field-trails\2025-11-05-Pig-Slurry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ED3D62F-47B5-469A-A226-7E546018DD55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF85691F-BE76-4693-94B8-7E2D63571FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -38,10 +38,19 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={AA1BF658-B979-4146-9A0E-C46AC07D3CE1}</author>
     <author>tc={1F78B895-D85C-4922-97A4-38A181EFBF3B}</author>
   </authors>
   <commentList>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{1F78B895-D85C-4922-97A4-38A181EFBF3B}">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{AA1BF658-B979-4146-9A0E-C46AC07D3CE1}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This colum follows the original plan during the experiment, but OSI and TH was switched on the actual day for logistical reasons</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="1" shapeId="0" xr:uid="{1F78B895-D85C-4922-97A4-38A181EFBF3B}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -528,6 +537,9 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="E1" dT="2026-03-12T08:15:27.29" personId="{DB2C1B22-E491-4202-AEFE-EDDF00FCCA1A}" id="{AA1BF658-B979-4146-9A0E-C46AC07D3CE1}">
+    <text>This colum follows the original plan during the experiment, but OSI and TH was switched on the actual day for logistical reasons</text>
+  </threadedComment>
   <threadedComment ref="I1" dT="2026-03-04T10:16:56.49" personId="{DB2C1B22-E491-4202-AEFE-EDDF00FCCA1A}" id="{1F78B895-D85C-4922-97A4-38A181EFBF3B}">
     <text>Time of slurry application in relation to the start of the experiment
 (bks simply corrected to use the 1st measurement point)</text>
@@ -608,7 +620,7 @@
         <v>0</v>
       </c>
       <c r="J2">
-        <f>(F2^0.5)*$L$2</f>
+        <f t="shared" ref="J2:J20" si="0">(F2^0.5)*$L$2</f>
         <v>34.571664698131038</v>
       </c>
       <c r="L2">
@@ -648,7 +660,7 @@
         <v>0</v>
       </c>
       <c r="J3">
-        <f>(F3^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>33.285131815872383</v>
       </c>
     </row>
@@ -672,14 +684,14 @@
         <v>0.4861111111111111</v>
       </c>
       <c r="H4" s="4">
-        <f t="shared" ref="H4:H20" si="0">G4-$G$2</f>
+        <f t="shared" ref="H4:H20" si="1">G4-$G$2</f>
         <v>0</v>
       </c>
       <c r="I4">
         <v>0</v>
       </c>
       <c r="J4">
-        <f>(F4^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>33.217465285599381</v>
       </c>
     </row>
@@ -711,7 +723,7 @@
         <v>0.4</v>
       </c>
       <c r="J5">
-        <f>(F5^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>33.231009614515173</v>
       </c>
     </row>
@@ -735,7 +747,7 @@
         <v>0.5083333333333333</v>
       </c>
       <c r="H6" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.2222222222222199E-2</v>
       </c>
       <c r="I6" s="5">
@@ -743,7 +755,7 @@
         <v>0.53333333333333333</v>
       </c>
       <c r="J6">
-        <f>(F6^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>33.231009614515173</v>
       </c>
     </row>
@@ -764,7 +776,7 @@
         <v>0.50277777777777777</v>
       </c>
       <c r="H7" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.6666666666666663E-2</v>
       </c>
       <c r="I7" s="5">
@@ -772,7 +784,7 @@
         <v>0.4</v>
       </c>
       <c r="J7">
-        <f>(F7^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>33.608034753612117</v>
       </c>
     </row>
@@ -796,7 +808,7 @@
         <v>0.50277777777777777</v>
       </c>
       <c r="H8" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.6666666666666663E-2</v>
       </c>
       <c r="I8" s="5">
@@ -804,7 +816,7 @@
         <v>0.4</v>
       </c>
       <c r="J8">
-        <f>(F8^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>34.047026301866659</v>
       </c>
     </row>
@@ -825,7 +837,7 @@
         <v>0.57777777777777772</v>
       </c>
       <c r="H9" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9.1666666666666619E-2</v>
       </c>
       <c r="I9" s="5">
@@ -833,7 +845,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="J9">
-        <f>(F9^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>33.79497003993346</v>
       </c>
     </row>
@@ -857,7 +869,7 @@
         <v>0.57152777777777775</v>
       </c>
       <c r="H10" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8.5416666666666641E-2</v>
       </c>
       <c r="I10">
@@ -865,7 +877,7 @@
         <v>2.0499999999999998</v>
       </c>
       <c r="J10">
-        <f>(F10^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>33.79497003993346</v>
       </c>
     </row>
@@ -889,7 +901,7 @@
         <v>0.58402777777777781</v>
       </c>
       <c r="H11" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9.7916666666666707E-2</v>
       </c>
       <c r="I11" s="5">
@@ -897,7 +909,7 @@
         <v>2.35</v>
       </c>
       <c r="J11">
-        <f>(F11^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>34.126236241343697</v>
       </c>
     </row>
@@ -918,7 +930,7 @@
         <v>0.58958333333333335</v>
       </c>
       <c r="H12" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.10347222222222224</v>
       </c>
       <c r="I12" s="5">
@@ -926,7 +938,7 @@
         <v>2.4833333333333334</v>
       </c>
       <c r="J12">
-        <f>(F12^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>33.054500450014373</v>
       </c>
     </row>
@@ -950,7 +962,7 @@
         <v>0.59513888888888888</v>
       </c>
       <c r="H13" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.10902777777777778</v>
       </c>
       <c r="I13" s="5">
@@ -958,7 +970,7 @@
         <v>2.6166666666666667</v>
       </c>
       <c r="J13">
-        <f>(F13^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>33.446972957204963</v>
       </c>
     </row>
@@ -982,7 +994,7 @@
         <v>0.60069444444444442</v>
       </c>
       <c r="H14" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.11458333333333331</v>
       </c>
       <c r="I14">
@@ -990,7 +1002,7 @@
         <v>2.75</v>
       </c>
       <c r="J14">
-        <f>(F14^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>33.541019662496851</v>
       </c>
     </row>
@@ -1011,7 +1023,7 @@
         <v>0.60624999999999996</v>
       </c>
       <c r="H15" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.12013888888888885</v>
       </c>
       <c r="I15" s="5">
@@ -1019,7 +1031,7 @@
         <v>2.8833333333333333</v>
       </c>
       <c r="J15">
-        <f>(F15^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>33.741665637605976</v>
       </c>
     </row>
@@ -1043,7 +1055,7 @@
         <v>0.6118055555555556</v>
       </c>
       <c r="H16" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.1256944444444445</v>
       </c>
       <c r="I16" s="5">
@@ -1051,7 +1063,7 @@
         <v>3.0166666666666666</v>
       </c>
       <c r="J16">
-        <f>(F16^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>35.887323667278395</v>
       </c>
     </row>
@@ -1075,7 +1087,7 @@
         <v>0.61736111111111114</v>
       </c>
       <c r="H17" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.13125000000000003</v>
       </c>
       <c r="I17" s="5">
@@ -1083,7 +1095,7 @@
         <v>3.15</v>
       </c>
       <c r="J17">
-        <f>(F17^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>35.887323667278395</v>
       </c>
     </row>
@@ -1104,7 +1116,7 @@
         <v>0.62291666666666667</v>
       </c>
       <c r="H18" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.13680555555555557</v>
       </c>
       <c r="I18" s="5">
@@ -1112,7 +1124,7 @@
         <v>3.2833333333333332</v>
       </c>
       <c r="J18">
-        <f>(F18^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>34.895558456628834</v>
       </c>
     </row>
@@ -1136,7 +1148,7 @@
         <v>0.62847222222222221</v>
       </c>
       <c r="H19" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.1423611111111111</v>
       </c>
       <c r="I19" s="5">
@@ -1144,7 +1156,7 @@
         <v>3.4166666666666665</v>
       </c>
       <c r="J19">
-        <f>(F19^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>33.460424384636852</v>
       </c>
     </row>
@@ -1168,7 +1180,7 @@
         <v>0.63402777777777775</v>
       </c>
       <c r="H20" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.14791666666666664</v>
       </c>
       <c r="I20">
@@ -1176,7 +1188,7 @@
         <v>3.55</v>
       </c>
       <c r="J20">
-        <f>(F20^0.5)*$L$2</f>
+        <f t="shared" si="0"/>
         <v>34.113047357279591</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Lab data treatment finished
Lab data treatment of either experiment done, waiting to output csv-files untill checks of results are performed
</commit_message>
<xml_diff>
--- a/Field-trails/2025-11-05-Pig-Slurry/DFC overview pig.xlsx
+++ b/Field-trails/2025-11-05-Pig-Slurry/DFC overview pig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Field-trails\2025-11-05-Pig-Slurry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF85691F-BE76-4693-94B8-7E2D63571FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEFAFD2F-6E46-439F-B9FA-E768F6DB269B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -197,7 +197,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -215,12 +215,6 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -244,13 +238,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -920,7 +915,7 @@
       <c r="D12">
         <v>9</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F12">

</xml_diff>